<commit_message>
Add pure iron results using the other group's measurements
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FwXsc2JBiGHJi72V8HsJjh
</commit_message>
<xml_diff>
--- a/report_hys/磁気ヒステリシス_データとグラフ.xlsx
+++ b/report_hys/磁気ヒステリシス_データとグラフ.xlsx
@@ -13,8 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="グラフ 空芯" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="グラフ アルニコ I-B" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="グラフ アルニコ B-H" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="透磁率曲線" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平行平板 V-x" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="グラフ 純鉄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="透磁率曲線" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平行平板 V-x" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1161,6 +1162,344 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
+            <v>(ⅰ) N 増加</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="4472C4"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$A$3:$A$16</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$B$3:$B$16</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>(ⅱ) N 減少</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="ED7D31"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="square"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="ED7D31"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="ED7D31"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$D$3:$D$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$E$3:$E$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>(ⅲ) S 増加</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="A5A5A5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="triangle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="A5A5A5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="A5A5A5"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$G$3:$G$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$H$3:$H$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>(ⅳ) S 減少</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="diamond"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFC000"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$J$3:$J$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$K$3:$K$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <v>(ⅴ) N 再び増加</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="x"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="5B9BD5"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$M$3:$M$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'グラフ 純鉄'!$N$3:$N$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>励磁電流 I [A]</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <numFmt formatCode="General" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+            <a:solidFill>
+              <a:srgbClr val="D9D9D9"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>磁束密度 B [T]</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <numFmt formatCode="General" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+            <a:solidFill>
+              <a:srgbClr val="D9D9D9"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+  <txPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="900">
+          <a:solidFill>
+            <a:srgbClr val="595959"/>
+          </a:solidFill>
+          <a:latin typeface="游ゴシック"/>
+          <a:ea typeface="游ゴシック"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ja-JP"/>
+    </a:p>
+  </txPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <roundedCorners val="0"/>
+  <style val="2"/>
+  <chart>
+    <autoTitleDeleted val="1"/>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
             <v>μ＝B/H</v>
           </tx>
           <spPr>
@@ -1411,6 +1750,33 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -3387,6 +3753,9 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
       <c r="C2">
         <f>A2*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3400,6 +3769,9 @@
       <c r="A3" t="n">
         <v>0.2</v>
       </c>
+      <c r="B3" t="n">
+        <v>0.13</v>
+      </c>
       <c r="C3">
         <f>A3*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3413,6 +3785,9 @@
       <c r="A4" t="n">
         <v>0.4</v>
       </c>
+      <c r="B4" t="n">
+        <v>0.3</v>
+      </c>
       <c r="C4">
         <f>A4*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3426,6 +3801,9 @@
       <c r="A5" t="n">
         <v>0.6</v>
       </c>
+      <c r="B5" t="n">
+        <v>0.33</v>
+      </c>
       <c r="C5">
         <f>A5*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3439,6 +3817,9 @@
       <c r="A6" t="n">
         <v>0.8</v>
       </c>
+      <c r="B6" t="n">
+        <v>0.48</v>
+      </c>
       <c r="C6">
         <f>A6*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3452,6 +3833,9 @@
       <c r="A7" t="n">
         <v>1</v>
       </c>
+      <c r="B7" t="n">
+        <v>0.51</v>
+      </c>
       <c r="C7">
         <f>A7*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3465,6 +3849,9 @@
       <c r="A8" t="n">
         <v>1.5</v>
       </c>
+      <c r="B8" t="n">
+        <v>0.62</v>
+      </c>
       <c r="C8">
         <f>A8*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3478,6 +3865,9 @@
       <c r="A9" t="n">
         <v>2</v>
       </c>
+      <c r="B9" t="n">
+        <v>0.73</v>
+      </c>
       <c r="C9">
         <f>A9*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3491,6 +3881,9 @@
       <c r="A10" t="n">
         <v>2.5</v>
       </c>
+      <c r="B10" t="n">
+        <v>0.82</v>
+      </c>
       <c r="C10">
         <f>A10*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3504,6 +3897,9 @@
       <c r="A11" t="n">
         <v>3</v>
       </c>
+      <c r="B11" t="n">
+        <v>0.9</v>
+      </c>
       <c r="C11">
         <f>A11*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3517,6 +3913,9 @@
       <c r="A12" t="n">
         <v>3.5</v>
       </c>
+      <c r="B12" t="n">
+        <v>0.98</v>
+      </c>
       <c r="C12">
         <f>A12*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3530,6 +3929,9 @@
       <c r="A13" t="n">
         <v>4</v>
       </c>
+      <c r="B13" t="n">
+        <v>1.02</v>
+      </c>
       <c r="C13">
         <f>A13*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3543,6 +3945,9 @@
       <c r="A14" t="n">
         <v>4.5</v>
       </c>
+      <c r="B14" t="n">
+        <v>1.09</v>
+      </c>
       <c r="C14">
         <f>A14*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3556,6 +3961,9 @@
       <c r="A15" t="n">
         <v>5</v>
       </c>
+      <c r="B15" t="n">
+        <v>1.13</v>
+      </c>
       <c r="C15">
         <f>A15*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3569,6 +3977,9 @@
       <c r="A16" t="n">
         <v>4.5</v>
       </c>
+      <c r="B16" t="n">
+        <v>1.1</v>
+      </c>
       <c r="C16">
         <f>A16*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3582,6 +3993,9 @@
       <c r="A17" t="n">
         <v>4</v>
       </c>
+      <c r="B17" t="n">
+        <v>1.08</v>
+      </c>
       <c r="C17">
         <f>A17*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3595,6 +4009,9 @@
       <c r="A18" t="n">
         <v>3.5</v>
       </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
       <c r="C18">
         <f>A18*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3608,6 +4025,9 @@
       <c r="A19" t="n">
         <v>3</v>
       </c>
+      <c r="B19" t="n">
+        <v>0.92</v>
+      </c>
       <c r="C19">
         <f>A19*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3621,6 +4041,9 @@
       <c r="A20" t="n">
         <v>2.5</v>
       </c>
+      <c r="B20" t="n">
+        <v>0.88</v>
+      </c>
       <c r="C20">
         <f>A20*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3634,6 +4057,9 @@
       <c r="A21" t="n">
         <v>2</v>
       </c>
+      <c r="B21" t="n">
+        <v>0.8</v>
+      </c>
       <c r="C21">
         <f>A21*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3647,6 +4073,9 @@
       <c r="A22" t="n">
         <v>1.5</v>
       </c>
+      <c r="B22" t="n">
+        <v>0.7</v>
+      </c>
       <c r="C22">
         <f>A22*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3660,6 +4089,9 @@
       <c r="A23" t="n">
         <v>1</v>
       </c>
+      <c r="B23" t="n">
+        <v>0.59</v>
+      </c>
       <c r="C23">
         <f>A23*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3673,6 +4105,9 @@
       <c r="A24" t="n">
         <v>0.5</v>
       </c>
+      <c r="B24" t="n">
+        <v>0.42</v>
+      </c>
       <c r="C24">
         <f>A24*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3686,6 +4121,9 @@
       <c r="A25" t="n">
         <v>0</v>
       </c>
+      <c r="B25" t="n">
+        <v>0.01</v>
+      </c>
       <c r="C25">
         <f>A25*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3699,6 +4137,9 @@
       <c r="A26" t="n">
         <v>-0.5</v>
       </c>
+      <c r="B26" t="n">
+        <v>-0.33</v>
+      </c>
       <c r="C26">
         <f>A26*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3712,6 +4153,9 @@
       <c r="A27" t="n">
         <v>-1</v>
       </c>
+      <c r="B27" t="n">
+        <v>-0.57</v>
+      </c>
       <c r="C27">
         <f>A27*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3725,6 +4169,9 @@
       <c r="A28" t="n">
         <v>-1.5</v>
       </c>
+      <c r="B28" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
       <c r="C28">
         <f>A28*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3738,6 +4185,9 @@
       <c r="A29" t="n">
         <v>-2</v>
       </c>
+      <c r="B29" t="n">
+        <v>-0.8</v>
+      </c>
       <c r="C29">
         <f>A29*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3751,6 +4201,9 @@
       <c r="A30" t="n">
         <v>-2.5</v>
       </c>
+      <c r="B30" t="n">
+        <v>-0.87</v>
+      </c>
       <c r="C30">
         <f>A30*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3764,6 +4217,9 @@
       <c r="A31" t="n">
         <v>-3</v>
       </c>
+      <c r="B31" t="n">
+        <v>-0.95</v>
+      </c>
       <c r="C31">
         <f>A31*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3777,6 +4233,9 @@
       <c r="A32" t="n">
         <v>-3.5</v>
       </c>
+      <c r="B32" t="n">
+        <v>-1.02</v>
+      </c>
       <c r="C32">
         <f>A32*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3790,6 +4249,9 @@
       <c r="A33" t="n">
         <v>-4</v>
       </c>
+      <c r="B33" t="n">
+        <v>-1.1</v>
+      </c>
       <c r="C33">
         <f>A33*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3803,6 +4265,9 @@
       <c r="A34" t="n">
         <v>-4.5</v>
       </c>
+      <c r="B34" t="n">
+        <v>-1.13</v>
+      </c>
       <c r="C34">
         <f>A34*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3816,6 +4281,9 @@
       <c r="A35" t="n">
         <v>-5</v>
       </c>
+      <c r="B35" t="n">
+        <v>-1.23</v>
+      </c>
       <c r="C35">
         <f>A35*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3829,6 +4297,9 @@
       <c r="A36" t="n">
         <v>-4.5</v>
       </c>
+      <c r="B36" t="n">
+        <v>-1.19</v>
+      </c>
       <c r="C36">
         <f>A36*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3842,6 +4313,9 @@
       <c r="A37" t="n">
         <v>-4</v>
       </c>
+      <c r="B37" t="n">
+        <v>-1.11</v>
+      </c>
       <c r="C37">
         <f>A37*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3855,6 +4329,9 @@
       <c r="A38" t="n">
         <v>-3.5</v>
       </c>
+      <c r="B38" t="n">
+        <v>-1.05</v>
+      </c>
       <c r="C38">
         <f>A38*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3868,6 +4345,9 @@
       <c r="A39" t="n">
         <v>-3</v>
       </c>
+      <c r="B39" t="n">
+        <v>-1</v>
+      </c>
       <c r="C39">
         <f>A39*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3881,6 +4361,9 @@
       <c r="A40" t="n">
         <v>-2.5</v>
       </c>
+      <c r="B40" t="n">
+        <v>-0.92</v>
+      </c>
       <c r="C40">
         <f>A40*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3894,6 +4377,9 @@
       <c r="A41" t="n">
         <v>-2</v>
       </c>
+      <c r="B41" t="n">
+        <v>-0.83</v>
+      </c>
       <c r="C41">
         <f>A41*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3907,6 +4393,9 @@
       <c r="A42" t="n">
         <v>-1.5</v>
       </c>
+      <c r="B42" t="n">
+        <v>-0.72</v>
+      </c>
       <c r="C42">
         <f>A42*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3920,6 +4409,9 @@
       <c r="A43" t="n">
         <v>-1</v>
       </c>
+      <c r="B43" t="n">
+        <v>-0.62</v>
+      </c>
       <c r="C43">
         <f>A43*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3933,6 +4425,9 @@
       <c r="A44" t="n">
         <v>-0.5</v>
       </c>
+      <c r="B44" t="n">
+        <v>-0.43</v>
+      </c>
       <c r="C44">
         <f>A44*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3946,6 +4441,9 @@
       <c r="A45" t="n">
         <v>0</v>
       </c>
+      <c r="B45" t="n">
+        <v>-0.05</v>
+      </c>
       <c r="C45">
         <f>A45*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3959,6 +4457,9 @@
       <c r="A46" t="n">
         <v>0.5</v>
       </c>
+      <c r="B46" t="n">
+        <v>0.23</v>
+      </c>
       <c r="C46">
         <f>A46*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3972,6 +4473,9 @@
       <c r="A47" t="n">
         <v>1</v>
       </c>
+      <c r="B47" t="n">
+        <v>0.52</v>
+      </c>
       <c r="C47">
         <f>A47*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3985,6 +4489,9 @@
       <c r="A48" t="n">
         <v>1.5</v>
       </c>
+      <c r="B48" t="n">
+        <v>0.67</v>
+      </c>
       <c r="C48">
         <f>A48*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -3998,6 +4505,9 @@
       <c r="A49" t="n">
         <v>2</v>
       </c>
+      <c r="B49" t="n">
+        <v>0.75</v>
+      </c>
       <c r="C49">
         <f>A49*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -4011,6 +4521,9 @@
       <c r="A50" t="n">
         <v>2.5</v>
       </c>
+      <c r="B50" t="n">
+        <v>0.83</v>
+      </c>
       <c r="C50">
         <f>A50*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -4024,6 +4537,9 @@
       <c r="A51" t="n">
         <v>3</v>
       </c>
+      <c r="B51" t="n">
+        <v>0.91</v>
+      </c>
       <c r="C51">
         <f>A51*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -4037,6 +4553,9 @@
       <c r="A52" t="n">
         <v>3.5</v>
       </c>
+      <c r="B52" t="n">
+        <v>0.99</v>
+      </c>
       <c r="C52">
         <f>A52*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -4050,6 +4569,9 @@
       <c r="A53" t="n">
         <v>4</v>
       </c>
+      <c r="B53" t="n">
+        <v>1.07</v>
+      </c>
       <c r="C53">
         <f>A53*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -4063,6 +4585,9 @@
       <c r="A54" t="n">
         <v>4.5</v>
       </c>
+      <c r="B54" t="n">
+        <v>1.12</v>
+      </c>
       <c r="C54">
         <f>A54*'空芯（換算式）'!$G$2</f>
         <v/>
@@ -4075,6 +4600,9 @@
     <row r="55">
       <c r="A55" t="n">
         <v>5</v>
+      </c>
+      <c r="B55" t="n">
+        <v>1.2</v>
       </c>
       <c r="C55">
         <f>A55*'空芯（換算式）'!$G$2</f>
@@ -5698,147 +6226,462 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>H [A/m]</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>μ [H/m]</t>
+          <t>(ⅰ) N 増加</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>(ⅱ) N 減少</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>(ⅲ) S 増加</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>(ⅳ) S 減少</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>(ⅴ) N 再び増加</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1779.86927797401</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2.809195069478025e-06</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>励磁電流 I [A]</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>B [T]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>励磁電流 I [A]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B [T]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>励磁電流 I [A]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>B [T]</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>励磁電流 I [A]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>B [T]</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>励磁電流 I [A]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>B [T]</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3559.738555948019</v>
+        <v>0</v>
       </c>
       <c r="B3" t="n">
-        <v>3.090114576425827e-06</v>
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-0.05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5339.607833922028</v>
+        <v>0.2</v>
       </c>
       <c r="B4" t="n">
-        <v>3.37103408337363e-06</v>
+        <v>0.13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>7119.477111896039</v>
+        <v>0.4</v>
       </c>
       <c r="B5" t="n">
-        <v>3.230574329899729e-06</v>
+        <v>0.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-4</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>8899.346389870048</v>
+        <v>0.6</v>
       </c>
       <c r="B6" t="n">
-        <v>3.483401886152751e-06</v>
+        <v>0.33</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-1.05</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.67</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>13349.01958480507</v>
+        <v>0.8</v>
       </c>
       <c r="B7" t="n">
-        <v>3.520857820412458e-06</v>
+        <v>0.48</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>17798.6927797401</v>
+        <v>1</v>
       </c>
       <c r="B8" t="n">
-        <v>3.651953590321432e-06</v>
+        <v>0.51</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.83</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>22248.36597467512</v>
+        <v>1.5</v>
       </c>
       <c r="B9" t="n">
-        <v>3.685663931155169e-06</v>
+        <v>0.62</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.91</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>26698.03916961014</v>
+        <v>2</v>
       </c>
       <c r="B10" t="n">
-        <v>3.445945951893044e-06</v>
+        <v>0.73</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="M10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.99</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>31147.71236454517</v>
+        <v>2.5</v>
       </c>
       <c r="B11" t="n">
-        <v>3.210508650832029e-06</v>
+        <v>0.82</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="M11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1.07</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>35597.38555948019</v>
+        <v>3</v>
       </c>
       <c r="B12" t="n">
-        <v>3.090114576425827e-06</v>
+        <v>0.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-1.13</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="M12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1.12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>40047.05875441521</v>
+        <v>3.5</v>
       </c>
       <c r="B13" t="n">
-        <v>3.995299654368747e-06</v>
+        <v>0.98</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="M13" t="n">
+        <v>5</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>44496.73194935024</v>
+        <v>4</v>
       </c>
       <c r="B14" t="n">
-        <v>4.719447716723081e-06</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>48946.40514428527</v>
+        <v>4.5</v>
       </c>
       <c r="B15" t="n">
-        <v>5.72054268693707e-06</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>53396.07833922029</v>
+        <v>5</v>
       </c>
       <c r="B16" t="n">
-        <v>7.11662750934433e-06</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>57845.75153415532</v>
-      </c>
-      <c r="B17" t="n">
-        <v>8.297930051381242e-06</v>
+        <v>1.13</v>
       </c>
     </row>
   </sheetData>
@@ -5853,6 +6696,161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>H [A/m]</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>μ [H/m]</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1779.86927797401</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2.809195069478025e-06</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3559.738555948019</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3.090114576425827e-06</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5339.607833922028</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3.37103408337363e-06</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>7119.477111896039</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3.230574329899729e-06</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>8899.346389870048</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3.483401886152751e-06</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>13349.01958480507</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3.520857820412458e-06</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>17798.6927797401</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3.651953590321432e-06</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>22248.36597467512</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3.685663931155169e-06</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>26698.03916961014</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3.445945951893044e-06</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>31147.71236454517</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3.210508650832029e-06</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>35597.38555948019</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3.090114576425827e-06</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>40047.05875441521</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3.995299654368747e-06</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>44496.73194935024</v>
+      </c>
+      <c r="B14" t="n">
+        <v>4.719447716723081e-06</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>48946.40514428527</v>
+      </c>
+      <c r="B15" t="n">
+        <v>5.72054268693707e-06</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>53396.07833922029</v>
+      </c>
+      <c r="B16" t="n">
+        <v>7.11662750934433e-06</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>57845.75153415532</v>
+      </c>
+      <c r="B17" t="n">
+        <v>8.297930051381242e-06</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>